<commit_message>
added all graphs files for histeretic
</commit_message>
<xml_diff>
--- a/SSW_CurvaCalibracion.xlsx
+++ b/SSW_CurvaCalibracion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pablo\Desktop\InvestigacionUSFQ\SSWCompleteAnalysis\SingleSolitaryWaveAnalysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3DE6784-D2DA-4039-B8EB-B9E43679B580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C69670CD-90A6-4C44-BB11-419F10EF381B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{2BD432D8-4488-4A89-A586-01F393994D8E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{2BD432D8-4488-4A89-A586-01F393994D8E}"/>
   </bookViews>
   <sheets>
     <sheet name="SSW_CalibrationCurve" sheetId="2" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="28">
   <si>
     <t>Archivo: SSW_GroupSimulationModel.m</t>
   </si>
@@ -147,9 +147,6 @@
     <t>k</t>
   </si>
   <si>
-    <t>Datos Matlab 0.3</t>
-  </si>
-  <si>
     <t>Datos Matlab 0.5</t>
   </si>
   <si>
@@ -169,6 +166,9 @@
   </si>
   <si>
     <t>k_ajustado</t>
+  </si>
+  <si>
+    <t>K - 0.3</t>
   </si>
 </sst>
 </file>
@@ -414,11 +414,11 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>K_values!$B$2</c:f>
+              <c:f>K_values!$B$13</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>K - 0.1</c:v>
+                  <c:v>K - 0.3</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -447,7 +447,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>K_values!$C$4:$C$11</c:f>
+              <c:f>K_values!$C$15:$C$22</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="8"/>
@@ -480,33 +480,33 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>K_values!$D$4:$D$11</c:f>
+              <c:f>K_values!$D$15:$D$22</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>1.4007381733822328</c:v>
+                  <c:v>1.3259736795022041</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.2140668286409155</c:v>
+                  <c:v>1.1531017802399695</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.1177048296059127</c:v>
+                  <c:v>1.0821813204036701</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.0909213561826436</c:v>
+                  <c:v>1.05394888195359</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.08058437749855</c:v>
+                  <c:v>1.0434829598242401</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.0723113034395499</c:v>
+                  <c:v>1.0350255733857601</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.0694334868948585</c:v>
+                  <c:v>1.0306193761935976</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.0629208338167233</c:v>
+                  <c:v>1.0245285302824279</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -600,34 +600,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="2">
-                  <c:v>1.911255690705151</c:v>
+                  <c:v>1.746240577829965</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.4725638452246448</c:v>
+                  <c:v>1.3337289319193049</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.3561559904511253</c:v>
+                  <c:v>1.2359819908382841</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.2023018139907831</c:v>
+                  <c:v>1.117990995419142</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.1392003263497481</c:v>
+                  <c:v>1.0746240577829964</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.1049107556644473</c:v>
+                  <c:v>1.0527671772980136</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.0889149485530791</c:v>
+                  <c:v>1.0430842198490353</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.0721872490315638</c:v>
+                  <c:v>1.0333728931919304</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.0629274673708604</c:v>
+                  <c:v>1.0282052426737605</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.0544051802451302</c:v>
+                  <c:v>1.0235981990838283</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2160,7 +2160,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80A9438D-FD9D-44C5-9D03-77FA3395C423}">
-  <dimension ref="B2:AD38"/>
+  <dimension ref="B2:AF38"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="3" width="8.796875" style="1"/>
@@ -2170,7 +2170,7 @@
     <col min="8" max="16384" width="8.796875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:30" x14ac:dyDescent="0.45">
+    <row r="2" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -2181,18 +2181,18 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="3" spans="2:30" x14ac:dyDescent="0.45">
-      <c r="X3" s="17" t="s">
+    <row r="3" spans="2:32" x14ac:dyDescent="0.45">
+      <c r="Z3" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="Y3" s="17"/>
-      <c r="Z3" s="17"/>
       <c r="AA3" s="17"/>
       <c r="AB3" s="17"/>
       <c r="AC3" s="17"/>
       <c r="AD3" s="17"/>
-    </row>
-    <row r="4" spans="2:30" x14ac:dyDescent="0.45">
+      <c r="AE3" s="17"/>
+      <c r="AF3" s="17"/>
+    </row>
+    <row r="4" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B4" s="17" t="s">
         <v>3</v>
       </c>
@@ -2202,29 +2202,40 @@
       <c r="F4" s="17"/>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
-      <c r="X4" s="3" t="s">
+      <c r="J4" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="K4" s="17"/>
+      <c r="L4" s="17"/>
+      <c r="M4" s="17"/>
+      <c r="N4" s="17"/>
+      <c r="O4" s="17"/>
+      <c r="P4" s="17"/>
+      <c r="Q4" s="17"/>
+      <c r="R4" s="17"/>
+      <c r="Z4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="Y4" s="4">
+      <c r="AA4" s="4">
         <v>10</v>
       </c>
-      <c r="Z4" s="4">
+      <c r="AB4" s="4">
         <v>100</v>
       </c>
-      <c r="AA4" s="4">
+      <c r="AC4" s="4">
         <v>300</v>
       </c>
-      <c r="AB4" s="4">
+      <c r="AD4" s="4">
         <v>500</v>
       </c>
-      <c r="AC4" s="4">
+      <c r="AE4" s="4">
         <v>700</v>
       </c>
-      <c r="AD4" s="3">
+      <c r="AF4" s="3">
         <v>1000</v>
       </c>
     </row>
-    <row r="5" spans="2:30" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B5" s="3" t="s">
         <v>4</v>
       </c>
@@ -2246,29 +2257,56 @@
       <c r="H5" s="3">
         <v>1000</v>
       </c>
-      <c r="X5" s="3">
+      <c r="J5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="K5" s="3">
+        <v>1</v>
+      </c>
+      <c r="L5" s="3">
+        <v>5</v>
+      </c>
+      <c r="M5" s="4">
+        <v>10</v>
+      </c>
+      <c r="N5" s="4">
+        <v>100</v>
+      </c>
+      <c r="O5" s="4">
+        <v>300</v>
+      </c>
+      <c r="P5" s="4">
+        <v>500</v>
+      </c>
+      <c r="Q5" s="4">
+        <v>700</v>
+      </c>
+      <c r="R5" s="3">
+        <v>1000</v>
+      </c>
+      <c r="Z5" s="3">
         <v>0.1</v>
       </c>
-      <c r="Y5" s="3">
+      <c r="AA5" s="3">
         <v>2.1252823576404498E-3</v>
       </c>
-      <c r="Z5" s="3">
+      <c r="AB5" s="3">
         <v>1.5349548257569E-3</v>
       </c>
-      <c r="AA5" s="3">
+      <c r="AC5" s="3">
         <v>1.2459906107288501E-3</v>
       </c>
-      <c r="AB5" s="3">
+      <c r="AD5" s="3">
         <v>1.13030798522664E-3</v>
       </c>
-      <c r="AC5" s="3">
+      <c r="AE5" s="3">
         <v>1.06244287429404E-3</v>
       </c>
-      <c r="AD5" s="5">
+      <c r="AF5" s="5">
         <v>9.978169398421491E-4</v>
       </c>
     </row>
-    <row r="6" spans="2:30" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
@@ -2296,15 +2334,50 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="X6" s="3"/>
-      <c r="Y6" s="3"/>
+      <c r="J6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="K6" s="4">
+        <f>LOG10(K5)</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="4">
+        <f>LOG10(L5)</f>
+        <v>0.69897000433601886</v>
+      </c>
+      <c r="M6" s="4">
+        <f>LOG10(M5)</f>
+        <v>1</v>
+      </c>
+      <c r="N6" s="4">
+        <f t="shared" ref="N6:R6" si="1">LOG10(N5)</f>
+        <v>2</v>
+      </c>
+      <c r="O6" s="4">
+        <f t="shared" si="1"/>
+        <v>2.4771212547196626</v>
+      </c>
+      <c r="P6" s="4">
+        <f t="shared" si="1"/>
+        <v>2.6989700043360187</v>
+      </c>
+      <c r="Q6" s="4">
+        <f t="shared" si="1"/>
+        <v>2.8450980400142569</v>
+      </c>
+      <c r="R6" s="4">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
       <c r="Z6" s="3"/>
       <c r="AA6" s="3"/>
       <c r="AB6" s="3"/>
       <c r="AC6" s="3"/>
-      <c r="AD6" s="5"/>
-    </row>
-    <row r="7" spans="2:30" x14ac:dyDescent="0.45">
+      <c r="AD6" s="3"/>
+      <c r="AE6" s="3"/>
+      <c r="AF6" s="5"/>
+    </row>
+    <row r="7" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B7" s="3">
         <v>0.1</v>
       </c>
@@ -2326,29 +2399,52 @@
       <c r="H7" s="7">
         <v>9.978169398421491E-4</v>
       </c>
-      <c r="X7" s="3">
+      <c r="J7" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="1">
+        <v>2.1867939205959799E-3</v>
+      </c>
+      <c r="N7" s="6">
+        <v>1.5349548257569E-3</v>
+      </c>
+      <c r="O7" s="6">
+        <v>1.2459906107288501E-3</v>
+      </c>
+      <c r="P7" s="6">
+        <v>1.13030798522664E-3</v>
+      </c>
+      <c r="Q7" s="6">
+        <v>1.06244287429404E-3</v>
+      </c>
+      <c r="R7" s="7">
+        <v>9.978169398421491E-4</v>
+      </c>
+      <c r="Z7" s="3">
         <v>0.3</v>
       </c>
-      <c r="Y7" s="3">
+      <c r="AA7" s="3">
         <v>2.15971893357225E-3</v>
       </c>
-      <c r="Z7" s="3">
+      <c r="AB7" s="3">
         <v>1.5245798642394099E-3</v>
       </c>
-      <c r="AA7" s="3">
+      <c r="AC7" s="3">
         <v>1.2349915672320801E-3</v>
       </c>
-      <c r="AB7" s="3">
+      <c r="AD7" s="3">
         <v>1.1210804794715E-3</v>
       </c>
-      <c r="AC7" s="3">
+      <c r="AE7" s="3">
         <v>1.0543159670394599E-3</v>
       </c>
-      <c r="AD7" s="5">
+      <c r="AF7" s="5">
         <v>9.8983598711006393E-4</v>
       </c>
     </row>
-    <row r="8" spans="2:30" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B8" s="3">
         <v>0.3</v>
       </c>
@@ -2370,29 +2466,54 @@
       <c r="H8" s="5">
         <v>9.8983598711006393E-4</v>
       </c>
-      <c r="X8" s="3">
+      <c r="J8" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3">
+        <v>2.3675139000000002E-3</v>
+      </c>
+      <c r="M8" s="3">
+        <v>2.15971893357225E-3</v>
+      </c>
+      <c r="N8" s="3">
+        <v>1.5245798642394099E-3</v>
+      </c>
+      <c r="O8" s="3">
+        <v>1.2349915672320801E-3</v>
+      </c>
+      <c r="P8" s="3">
+        <v>1.1210804794715E-3</v>
+      </c>
+      <c r="Q8" s="3">
+        <v>1.0543159670394599E-3</v>
+      </c>
+      <c r="R8" s="5">
+        <v>9.8983598711006393E-4</v>
+      </c>
+      <c r="Z8" s="3">
         <v>0.5</v>
       </c>
-      <c r="Y8" s="3">
+      <c r="AA8" s="3">
         <v>2.14970508462505E-3</v>
       </c>
-      <c r="Z8" s="3">
+      <c r="AB8" s="3">
         <v>1.4839440203368701E-3</v>
       </c>
-      <c r="AA8" s="3">
+      <c r="AC8" s="3">
         <v>1.19766476738336E-3</v>
       </c>
-      <c r="AB8" s="3">
+      <c r="AD8" s="3">
         <v>1.0891446262729801E-3</v>
       </c>
-      <c r="AC8" s="3">
+      <c r="AE8" s="3">
         <v>1.02655644409088E-3</v>
       </c>
-      <c r="AD8" s="5">
+      <c r="AF8" s="5">
         <v>9.6648717426287402E-4</v>
       </c>
     </row>
-    <row r="9" spans="2:30" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B9" s="3">
         <v>0.5</v>
       </c>
@@ -2414,8 +2535,31 @@
       <c r="H9" s="5">
         <v>9.6648717426287402E-4</v>
       </c>
-    </row>
-    <row r="11" spans="2:30" x14ac:dyDescent="0.45">
+      <c r="J9" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3">
+        <v>2.14970508462505E-3</v>
+      </c>
+      <c r="N9" s="3">
+        <v>1.4839440203368701E-3</v>
+      </c>
+      <c r="O9" s="3">
+        <v>1.19766476738336E-3</v>
+      </c>
+      <c r="P9" s="3">
+        <v>1.0891446262729801E-3</v>
+      </c>
+      <c r="Q9" s="3">
+        <v>1.02655644409088E-3</v>
+      </c>
+      <c r="R9" s="5">
+        <v>9.6648717426287402E-4</v>
+      </c>
+    </row>
+    <row r="11" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B11" s="18" t="s">
         <v>6</v>
       </c>
@@ -2432,7 +2576,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="2:30" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B12" s="18" t="s">
         <v>7</v>
       </c>
@@ -2451,13 +2595,13 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="2:30" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
     </row>
-    <row r="14" spans="2:30" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B14" s="17" t="s">
         <v>8</v>
       </c>
@@ -2468,33 +2612,33 @@
       <c r="G14" s="17"/>
       <c r="H14" s="17"/>
     </row>
-    <row r="15" spans="2:30" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B15" s="3">
         <f ca="1">D11</f>
         <v>0.34</v>
       </c>
       <c r="C15" s="3">
-        <f t="shared" ref="C15:H15" ca="1" si="1">_xlfn.FORECAST.LINEAR($D$11,C7:C8,$B$7:$B$8)</f>
+        <f t="shared" ref="C15:H15" ca="1" si="2">_xlfn.FORECAST.LINEAR($D$11,C7:C8,$B$7:$B$8)</f>
         <v>2.154303936167504E-3</v>
       </c>
       <c r="D15" s="3">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v>1.522504871935912E-3</v>
       </c>
       <c r="E15" s="3">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v>1.2327917585327262E-3</v>
       </c>
       <c r="F15" s="3">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v>1.1192349783204721E-3</v>
       </c>
       <c r="G15" s="3">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v>1.052690585588544E-3</v>
       </c>
       <c r="H15" s="3">
-        <f t="shared" ca="1" si="1"/>
+        <f t="shared" ca="1" si="2"/>
         <v>9.8823979656364699E-4</v>
       </c>
     </row>
@@ -2803,10 +2947,10 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B18:C18"/>
-    <mergeCell ref="X3:AD3"/>
+    <mergeCell ref="Z3:AF3"/>
     <mergeCell ref="B4:H4"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B12:C12"/>
@@ -2815,6 +2959,7 @@
     <mergeCell ref="E21:G21"/>
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="F12:G12"/>
+    <mergeCell ref="J4:R4"/>
   </mergeCells>
   <conditionalFormatting sqref="C15:H15">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
@@ -2832,7 +2977,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D0AE93B-6E63-4919-B10E-28F208192998}">
-  <dimension ref="B2:N33"/>
+  <dimension ref="B2:O33"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="9.06640625" style="10"/>
@@ -2843,31 +2988,31 @@
     <col min="11" max="16384" width="9.06640625" style="10"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" ht="15.75" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:15" ht="15.75" x14ac:dyDescent="0.5">
       <c r="B2" s="19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2" s="19"/>
       <c r="D2" s="19"/>
       <c r="G2" s="20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H2" s="20"/>
       <c r="I2" s="20"/>
       <c r="J2" s="20"/>
     </row>
-    <row r="3" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B3" s="11" t="s">
         <v>18</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B4" s="13">
         <v>10000000</v>
       </c>
@@ -2879,13 +3024,13 @@
         <v>1.4007381733822328</v>
       </c>
       <c r="L4" s="14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M4">
-        <v>0.91500000000000004</v>
-      </c>
-    </row>
-    <row r="5" spans="2:14" x14ac:dyDescent="0.45">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="5" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B5" s="13">
         <v>40000000</v>
       </c>
@@ -2897,13 +3042,13 @@
         <v>1.2140668286409155</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="M5" s="10">
-        <v>0.40799999999999997</v>
-      </c>
-    </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.45">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B6" s="13">
         <v>100000000</v>
       </c>
@@ -2915,7 +3060,7 @@
         <v>1.1177048296059127</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B7" s="13">
         <v>200000000</v>
       </c>
@@ -2927,13 +3072,13 @@
         <v>1.0909213561826436</v>
       </c>
       <c r="M7" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N7" s="15" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.45">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B8" s="13">
         <v>300000000</v>
       </c>
@@ -2947,7 +3092,7 @@
       <c r="M8" s="13"/>
       <c r="N8" s="15"/>
     </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B9" s="13">
         <v>500000000</v>
       </c>
@@ -2961,7 +3106,7 @@
       <c r="M9" s="13"/>
       <c r="N9" s="15"/>
     </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B10" s="13">
         <v>700000000</v>
       </c>
@@ -2977,10 +3122,14 @@
       </c>
       <c r="N10" s="15">
         <f t="shared" ref="N10:N11" si="1">1+$M$4*(M10/(1-0.1^2))^-$M$5</f>
-        <v>1.911255690705151</v>
-      </c>
-    </row>
-    <row r="11" spans="2:14" x14ac:dyDescent="0.45">
+        <v>1.746240577829965</v>
+      </c>
+      <c r="O10" s="10">
+        <f>M10*1000000</f>
+        <v>1000000</v>
+      </c>
+    </row>
+    <row r="11" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B11" s="13">
         <v>1000000000</v>
       </c>
@@ -2996,10 +3145,14 @@
       </c>
       <c r="N11" s="15">
         <f t="shared" si="1"/>
-        <v>1.4725638452246448</v>
-      </c>
-    </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.45">
+        <v>1.3337289319193049</v>
+      </c>
+      <c r="O11" s="10">
+        <f>M11*1000000</f>
+        <v>5000000</v>
+      </c>
+    </row>
+    <row r="12" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
       <c r="D12" s="12"/>
@@ -3008,12 +3161,12 @@
       </c>
       <c r="N12" s="15">
         <f>1+$M$4*(M12/(1-0.1^2))^-$M$5</f>
-        <v>1.3561559904511253</v>
-      </c>
-    </row>
-    <row r="13" spans="2:14" ht="15.75" x14ac:dyDescent="0.5">
+        <v>1.2359819908382841</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" ht="15.75" x14ac:dyDescent="0.5">
       <c r="B13" s="19" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="C13" s="19"/>
       <c r="D13" s="19"/>
@@ -3022,15 +3175,15 @@
       </c>
       <c r="N13" s="15">
         <f t="shared" ref="N13:N19" si="2">1+$M$4*(M13/(1-0.1^2))^-$M$5</f>
-        <v>1.2023018139907831</v>
-      </c>
-    </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.45">
+        <v>1.117990995419142</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B14" s="11" t="s">
         <v>18</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>19</v>
@@ -3040,10 +3193,10 @@
       </c>
       <c r="N14" s="15">
         <f t="shared" si="2"/>
-        <v>1.1392003263497481</v>
-      </c>
-    </row>
-    <row r="15" spans="2:14" x14ac:dyDescent="0.45">
+        <v>1.0746240577829964</v>
+      </c>
+    </row>
+    <row r="15" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B15" s="13">
         <v>10000000</v>
       </c>
@@ -3059,10 +3212,10 @@
       </c>
       <c r="N15" s="15">
         <f t="shared" si="2"/>
-        <v>1.1049107556644473</v>
-      </c>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.45">
+        <v>1.0527671772980136</v>
+      </c>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B16" s="13">
         <v>40000000</v>
       </c>
@@ -3078,7 +3231,7 @@
       </c>
       <c r="N16" s="15">
         <f t="shared" si="2"/>
-        <v>1.0889149485530791</v>
+        <v>1.0430842198490353</v>
       </c>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.45">
@@ -3097,7 +3250,7 @@
       </c>
       <c r="N17" s="15">
         <f t="shared" si="2"/>
-        <v>1.0721872490315638</v>
+        <v>1.0333728931919304</v>
       </c>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.45">
@@ -3116,7 +3269,7 @@
       </c>
       <c r="N18" s="15">
         <f t="shared" si="2"/>
-        <v>1.0629274673708604</v>
+        <v>1.0282052426737605</v>
       </c>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.45">
@@ -3135,7 +3288,7 @@
       </c>
       <c r="N19" s="15">
         <f t="shared" si="2"/>
-        <v>1.0544051802451302</v>
+        <v>1.0235981990838283</v>
       </c>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.45">
@@ -3181,7 +3334,7 @@
     </row>
     <row r="24" spans="2:14" ht="15.75" x14ac:dyDescent="0.5">
       <c r="B24" s="19" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C24" s="19"/>
       <c r="D24" s="19"/>
@@ -3191,7 +3344,7 @@
         <v>18</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D25" s="11" t="s">
         <v>19</v>
@@ -3301,6 +3454,7 @@
     <mergeCell ref="G2:J2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
changes histeric to defomration and strain
</commit_message>
<xml_diff>
--- a/SSW_CurvaCalibracion.xlsx
+++ b/SSW_CurvaCalibracion.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pablo\Desktop\InvestigacionUSFQ\SSWCompleteAnalysis\SingleSolitaryWaveAnalysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53EE8B61-2F2E-481E-ACA4-1B36FA4DD364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40F410CA-E299-4D45-B79F-D91BFC1A7EBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{2BD432D8-4488-4A89-A586-01F393994D8E}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{2BD432D8-4488-4A89-A586-01F393994D8E}"/>
   </bookViews>
   <sheets>
     <sheet name="SSW_CalibrationCurve" sheetId="2" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="32">
   <si>
     <t>Archivo: SSW_GroupSimulationModel.m</t>
   </si>
@@ -169,6 +169,18 @@
   </si>
   <si>
     <t>K - 0.3</t>
+  </si>
+  <si>
+    <t>0.1Mpa</t>
+  </si>
+  <si>
+    <t>0.01Mpa</t>
+  </si>
+  <si>
+    <t>0.001MPa</t>
+  </si>
+  <si>
+    <t>0.0001MPa</t>
   </si>
 </sst>
 </file>
@@ -299,7 +311,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
@@ -339,6 +351,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2594,12 +2607,27 @@
         <f t="array" aca="1" ref="H12" ca="1">IF(MAX(IF(C15:H15 &gt; D12, COLUMN(C15:H15)-COLUMN(C15)+1, 0))=0,3,MAX(IF(C15:H15 &gt; D12, COLUMN(C15:H15)-COLUMN(C15)+1, 0))+2)</f>
         <v>6</v>
       </c>
+      <c r="L12" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="M12" s="21" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="13" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
+      <c r="K13" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="L13" s="1">
+        <v>2.4086954999999999E-3</v>
+      </c>
+      <c r="M13" s="1">
+        <v>1.75</v>
+      </c>
     </row>
     <row r="14" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B14" s="17" t="s">
@@ -2611,6 +2639,15 @@
       <c r="F14" s="17"/>
       <c r="G14" s="17"/>
       <c r="H14" s="17"/>
+      <c r="K14" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="L14" s="1">
+        <v>3.6903573000000001E-3</v>
+      </c>
+      <c r="M14" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B15" s="3">
@@ -2641,8 +2678,17 @@
         <f t="shared" ca="1" si="2"/>
         <v>9.8823979656364699E-4</v>
       </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="K15" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="L15" s="1">
+        <v>1.5500348999999999E-3</v>
+      </c>
+      <c r="M15" s="1">
+        <v>3.35</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B17" s="17" t="s">
         <v>9</v>
       </c>
@@ -2651,8 +2697,17 @@
       <c r="E17" s="17"/>
       <c r="F17" s="17"/>
       <c r="G17" s="17"/>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="K17" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="L17" s="1">
+        <v>2.4463623000000002E-3</v>
+      </c>
+      <c r="M17" s="1">
+        <v>1.75</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B18" s="17" t="s">
         <v>10</v>
       </c>
@@ -2671,8 +2726,28 @@
         <f ca="1">10^(_xlfn.FORECAST.LINEAR($D$12,INDEX(6:6, H12):INDEX(6:6, H12+1),INDEX(15:15, H12):INDEX(15:15, H12+1)))</f>
         <v>597.4918815671075</v>
       </c>
-    </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="K18" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="L18" s="1">
+        <v>3.8038566000000002E-3</v>
+      </c>
+      <c r="M18" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="K20" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="L20" s="1">
+        <v>3.8302898E-3</v>
+      </c>
+      <c r="M20" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B21" s="16" t="s">
         <v>11</v>
       </c>
@@ -2683,7 +2758,7 @@
       <c r="F21" s="16"/>
       <c r="G21" s="16"/>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B22" s="3" t="s">
         <v>7</v>
       </c>
@@ -2699,8 +2774,17 @@
       <c r="G22" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="K22" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="L22" s="1">
+        <v>3.8360415999999999E-3</v>
+      </c>
+      <c r="M22" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B23" s="3">
         <v>1.8476923377406251E-3</v>
       </c>
@@ -2717,7 +2801,7 @@
         <v>14.374990072243435</v>
       </c>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B24" s="3">
         <v>1.7318046576407415E-3</v>
       </c>
@@ -2734,7 +2818,7 @@
         <v>5.7366344617829391E-2</v>
       </c>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B25" s="3">
         <v>1.6601886755722717E-3</v>
       </c>
@@ -2751,7 +2835,7 @@
         <v>21.807492181111002</v>
       </c>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B26" s="3">
         <v>2.656301880895029E-3</v>
       </c>
@@ -2768,7 +2852,7 @@
         <v>3.0456193140208896</v>
       </c>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B27" s="3">
         <v>3.093810425986021E-3</v>
       </c>
@@ -2785,14 +2869,14 @@
         <v>40.189987871759591</v>
       </c>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B29" s="3">
         <v>1.6211254126045442E-3</v>
       </c>
@@ -2809,7 +2893,7 @@
         <v>1647.1172015370512</v>
       </c>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B30" s="3">
         <v>1.5820621496551723E-3</v>
       </c>
@@ -2826,7 +2910,7 @@
         <v>805.32052067017969</v>
       </c>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="31" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B31" s="3">
         <v>1.7422215277640874E-3</v>
       </c>
@@ -2843,7 +2927,7 @@
         <v>22.034003152339405</v>
       </c>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B32" s="3">
         <v>2.5625500498065888E-3</v>
       </c>

</xml_diff>

<commit_message>
Complete Graphs for Pasta Mortero. Pending Review with JP.
</commit_message>
<xml_diff>
--- a/SSW_CurvaCalibracion.xlsx
+++ b/SSW_CurvaCalibracion.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pablo\Desktop\InvestigacionUSFQ\SSWCompleteAnalysis\SingleSolitaryWaveAnalysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{833C0986-B93B-42E5-A7F3-E9CEEDFB5440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{183DB95F-24AD-4F91-B687-735AA29AEF55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{2BD432D8-4488-4A89-A586-01F393994D8E}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="35">
   <si>
     <t>Archivo: SSW_GroupSimulationModel.m</t>
   </si>
@@ -183,14 +183,24 @@
   <si>
     <t>Mortero</t>
   </si>
+  <si>
+    <t>0p30</t>
+  </si>
+  <si>
+    <t>0p35</t>
+  </si>
+  <si>
+    <t>0p40</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.00000"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -312,7 +322,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
@@ -338,13 +348,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -353,6 +364,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -497,7 +509,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>2.4086954999999999E-3</c:v>
+                  <c:v>3.6903573000000001E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>1.5245798642394099E-3</c:v>
@@ -548,6 +560,152 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-1EAD-4AA4-8D47-80FD66777F4A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'SSW_CalibrationCurve (2)'!$E$23</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2.5586437235105598E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'SSW_CalibrationCurve (2)'!$G$23</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>3.467614180219901</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-1FB9-4DFA-B9B0-A29027BAC4F9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'SSW_CalibrationCurve (2)'!$C$9:$H$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>3.6403573E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.4839440203368701E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.19766476738336E-3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.0891446262729801E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.02655644409088E-3</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="0.000000">
+                  <c:v>9.6648717426287402E-4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'SSW_CalibrationCurve (2)'!$C$5:$H$5</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="General">
+                  <c:v>1000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-1FB9-4DFA-B9B0-A29027BAC4F9}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2345,16 +2503,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>322170</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>43143</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>249330</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>82364</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>21</xdr:col>
-      <xdr:colOff>501464</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>96931</xdr:rowOff>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>386602</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>151280</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -3121,7 +3279,7 @@
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="3" width="8.796875" style="1"/>
-    <col min="4" max="4" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.796875" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="8.796875" style="1"/>
     <col min="7" max="7" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="8.796875" style="1"/>
@@ -3139,37 +3297,37 @@
       </c>
     </row>
     <row r="3" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="Z3" s="18" t="s">
+      <c r="Z3" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="AA3" s="18"/>
-      <c r="AB3" s="18"/>
-      <c r="AC3" s="18"/>
-      <c r="AD3" s="18"/>
-      <c r="AE3" s="18"/>
-      <c r="AF3" s="18"/>
+      <c r="AA3" s="19"/>
+      <c r="AB3" s="19"/>
+      <c r="AC3" s="19"/>
+      <c r="AD3" s="19"/>
+      <c r="AE3" s="19"/>
+      <c r="AF3" s="19"/>
     </row>
     <row r="4" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="J4" s="18" t="s">
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="J4" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
-      <c r="N4" s="18"/>
-      <c r="O4" s="18"/>
-      <c r="P4" s="18"/>
-      <c r="Q4" s="18"/>
-      <c r="R4" s="18"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
       <c r="Z4" s="3" t="s">
         <v>4</v>
       </c>
@@ -3339,7 +3497,7 @@
         <v>0.1</v>
       </c>
       <c r="C7" s="1">
-        <v>3.6903573000000001E-3</v>
+        <v>3.7203573000000002E-3</v>
       </c>
       <c r="D7" s="6">
         <v>1.5349548257569E-3</v>
@@ -3406,7 +3564,7 @@
         <v>0.3</v>
       </c>
       <c r="C8" s="3">
-        <v>2.4086954999999999E-3</v>
+        <v>3.6903573000000001E-3</v>
       </c>
       <c r="D8" s="3">
         <v>1.5245798642394099E-3</v>
@@ -3472,8 +3630,8 @@
       <c r="B9" s="3">
         <v>0.5</v>
       </c>
-      <c r="C9" s="3">
-        <v>3.6903573000000001E-3</v>
+      <c r="C9" s="17">
+        <v>3.6403573E-3</v>
       </c>
       <c r="D9" s="3">
         <v>1.4839440203368701E-3</v>
@@ -3515,39 +3673,42 @@
       </c>
     </row>
     <row r="11" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="19"/>
+      <c r="C11" s="18"/>
       <c r="D11" s="3" cm="1">
         <f t="array" aca="1" ref="D11" ca="1">INDIRECT("F" &amp; H11)</f>
-        <v>0.3</v>
-      </c>
-      <c r="F11" s="19" t="s">
+        <v>0.5</v>
+      </c>
+      <c r="F11" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="19"/>
+      <c r="G11" s="18"/>
       <c r="H11" s="3">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="19"/>
+      <c r="C12" s="18"/>
       <c r="D12" s="5" cm="1">
         <f t="array" aca="1" ref="D12" ca="1">INDIRECT("E" &amp; H11)</f>
-        <v>2.9297447215697048E-3</v>
+        <v>3.4961620344202199E-3</v>
       </c>
       <c r="E12" s="8"/>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="G12" s="19"/>
+      <c r="G12" s="18"/>
       <c r="H12" s="3" cm="1">
         <f t="array" aca="1" ref="H12" ca="1">IF(MAX(IF(C15:H15 &gt; D12, COLUMN(C15:H15)-COLUMN(C15)+1, 0))=0,3,MAX(IF(C15:H15 &gt; D12, COLUMN(C15:H15)-COLUMN(C15)+1, 0))+2)</f>
         <v>3</v>
+      </c>
+      <c r="K12" s="1">
+        <v>0.3</v>
       </c>
       <c r="L12" s="16" t="s">
         <v>7</v>
@@ -3572,15 +3733,15 @@
       </c>
     </row>
     <row r="14" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
       <c r="K14" s="16" t="s">
         <v>27</v>
       </c>
@@ -3594,31 +3755,31 @@
     <row r="15" spans="2:32" x14ac:dyDescent="0.45">
       <c r="B15" s="3">
         <f ca="1">D11</f>
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="C15" s="3">
         <f t="shared" ref="C15:H15" ca="1" si="2">_xlfn.FORECAST.LINEAR($D$11,C7:C8,$B$7:$B$8)</f>
-        <v>2.4086955000000004E-3</v>
+        <v>3.6603572999999996E-3</v>
       </c>
       <c r="D15" s="3">
         <f t="shared" ca="1" si="2"/>
-        <v>1.5245798642394099E-3</v>
+        <v>1.5142049027219199E-3</v>
       </c>
       <c r="E15" s="3">
         <f t="shared" ca="1" si="2"/>
-        <v>1.2349915672320803E-3</v>
+        <v>1.22399252373531E-3</v>
       </c>
       <c r="F15" s="3">
         <f t="shared" ca="1" si="2"/>
-        <v>1.1210804794715003E-3</v>
+        <v>1.1118529737163601E-3</v>
       </c>
       <c r="G15" s="3">
         <f t="shared" ca="1" si="2"/>
-        <v>1.0543159670394599E-3</v>
+        <v>1.0461890597848798E-3</v>
       </c>
       <c r="H15" s="3">
         <f t="shared" ca="1" si="2"/>
-        <v>9.8983598711006393E-4</v>
+        <v>9.8185503437797899E-4</v>
       </c>
       <c r="K15" s="16" t="s">
         <v>27</v>
@@ -3631,14 +3792,14 @@
       </c>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="19"/>
       <c r="K17" s="16" t="s">
         <v>28</v>
       </c>
@@ -3650,13 +3811,13 @@
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="18"/>
+      <c r="C18" s="19"/>
       <c r="D18" s="9">
         <f ca="1">10^(_xlfn.FORECAST.LINEAR(D12,C6:D6,C15:D15))</f>
-        <v>1.7059436714625866E-3</v>
+        <v>0.16963693563959908</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>4</v>
@@ -3666,7 +3827,7 @@
       </c>
       <c r="G18" s="9">
         <f ca="1">10^(_xlfn.FORECAST.LINEAR($D$12,INDEX(6:6, H12):INDEX(6:6, H12+1),INDEX(15:15, H12):INDEX(15:15, H12+1)))</f>
-        <v>1.7059436714625866E-3</v>
+        <v>0.16963693563959908</v>
       </c>
       <c r="K18" s="16" t="s">
         <v>28</v>
@@ -3690,23 +3851,13 @@
       </c>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B21" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="C21" s="17"/>
-      <c r="E21" s="17" t="s">
+      <c r="E21" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B22" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="E22" s="3" t="s">
         <v>7</v>
       </c>
@@ -3727,212 +3878,128 @@
       </c>
     </row>
     <row r="23" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B23" s="3">
-        <v>1.8476923377406251E-3</v>
-      </c>
-      <c r="C23" s="3">
-        <v>32.625908938905432</v>
-      </c>
-      <c r="E23" s="3">
-        <v>3.4375671399828902E-3</v>
+      <c r="D23" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E23" s="23">
+        <v>2.5586437235105598E-3</v>
       </c>
       <c r="F23" s="3">
-        <v>0.3</v>
-      </c>
-      <c r="G23" s="3"/>
+        <v>0.5</v>
+      </c>
+      <c r="G23" s="3">
+        <v>3.467614180219901</v>
+      </c>
     </row>
     <row r="24" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B24" s="3">
-        <v>1.7318046576407415E-3</v>
-      </c>
-      <c r="C24" s="3">
-        <v>50.23345741286181</v>
-      </c>
-      <c r="E24" s="3">
-        <v>2.9297447215697048E-3</v>
+      <c r="D24" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24" s="23">
+        <v>3.3203773511161199E-3</v>
       </c>
       <c r="F24" s="3">
-        <v>0.3</v>
-      </c>
-      <c r="G24" s="3"/>
+        <v>0.5</v>
+      </c>
+      <c r="G24" s="3">
+        <v>0.29870404899774289</v>
+      </c>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B25" s="3">
-        <v>1.6601886755722717E-3</v>
-      </c>
-      <c r="C25" s="3">
-        <v>65.587469744581185</v>
-      </c>
-      <c r="E25" s="3">
-        <v>2.8906814586235896E-3</v>
+      <c r="D25" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E25" s="23">
+        <v>3.4961620344202199E-3</v>
       </c>
       <c r="F25" s="3">
-        <v>0.3</v>
-      </c>
-      <c r="G25" s="3"/>
+        <v>0.5</v>
+      </c>
+      <c r="G25" s="3">
+        <v>0.16963693563959908</v>
+      </c>
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B26" s="3">
-        <v>2.656301880895029E-3</v>
-      </c>
-      <c r="C26" s="3">
-        <v>1.606058593920398</v>
-      </c>
-      <c r="E26" s="3">
-        <v>2.7344284068107072E-3</v>
-      </c>
-      <c r="F26" s="3">
-        <v>0.3</v>
-      </c>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
       <c r="G26" s="3"/>
     </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B27" s="3">
-        <v>3.093810425986021E-3</v>
-      </c>
-      <c r="C27" s="3">
-        <v>0.31488993954243338</v>
-      </c>
-      <c r="E27" s="3">
-        <v>2.5977069864779878E-3</v>
-      </c>
-      <c r="F27" s="3">
-        <v>0.3</v>
-      </c>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
       <c r="G27" s="3"/>
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="E28" s="3">
-        <v>2.5586437235176618E-3</v>
-      </c>
-      <c r="F28" s="3">
-        <v>0.3</v>
-      </c>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
       <c r="G28" s="3"/>
     </row>
     <row r="29" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B29" s="3">
-        <v>1.6211254126045442E-3</v>
-      </c>
-      <c r="C29" s="3">
-        <v>75.857701690571744</v>
-      </c>
-      <c r="E29" s="3">
-        <v>2.5586437235105564E-3</v>
-      </c>
-      <c r="F29" s="3">
-        <v>0.3</v>
-      </c>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
       <c r="G29" s="3"/>
     </row>
     <row r="30" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B30" s="3">
-        <v>1.5820621496551723E-3</v>
-      </c>
-      <c r="C30" s="3">
-        <v>87.736132035461452</v>
-      </c>
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
     </row>
     <row r="31" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B31" s="3">
-        <v>1.7422215277640874E-3</v>
-      </c>
-      <c r="C31" s="3">
-        <v>48.322054338171974</v>
-      </c>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
     </row>
     <row r="32" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B32" s="3">
-        <v>2.5625500498065888E-3</v>
-      </c>
-      <c r="C32" s="3">
-        <v>2.2771441006533286</v>
-      </c>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
     </row>
-    <row r="33" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
+    <row r="33" spans="5:7" x14ac:dyDescent="0.45">
       <c r="E33" s="3"/>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
     </row>
-    <row r="34" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B34" s="3">
-        <v>1.2070548252907543E-3</v>
-      </c>
-      <c r="C34" s="3">
-        <v>370.78150112778985</v>
-      </c>
+    <row r="34" spans="5:7" x14ac:dyDescent="0.45">
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
     </row>
-    <row r="35" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B35" s="3">
-        <v>1.4414344030157622E-3</v>
-      </c>
-      <c r="C35" s="3">
-        <v>148.8424139248626</v>
-      </c>
+    <row r="35" spans="5:7" x14ac:dyDescent="0.45">
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
     </row>
-    <row r="36" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B36" s="3">
-        <v>2.027383347330769E-3</v>
-      </c>
-      <c r="C36" s="3">
-        <v>16.708602347103685</v>
-      </c>
+    <row r="36" spans="5:7" x14ac:dyDescent="0.45">
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
     </row>
-    <row r="37" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B37" s="3">
-        <v>2.3555147561467038E-3</v>
-      </c>
-      <c r="C37" s="3">
-        <v>4.9230945106328168</v>
-      </c>
+    <row r="37" spans="5:7" x14ac:dyDescent="0.45">
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="11">
     <mergeCell ref="B14:H14"/>
     <mergeCell ref="B17:G17"/>
     <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B21:C21"/>
     <mergeCell ref="E21:G21"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="F12:G12"/>
     <mergeCell ref="Z3:AF3"/>
     <mergeCell ref="B4:H4"/>
     <mergeCell ref="J4:R4"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="F11:G11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="F12:G12"/>
   </mergeCells>
   <conditionalFormatting sqref="C15:H15">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="greaterThan">
       <formula>$D$12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E23:E37">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>$D$12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3965,37 +4032,37 @@
       </c>
     </row>
     <row r="3" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="Z3" s="18" t="s">
+      <c r="Z3" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="AA3" s="18"/>
-      <c r="AB3" s="18"/>
-      <c r="AC3" s="18"/>
-      <c r="AD3" s="18"/>
-      <c r="AE3" s="18"/>
-      <c r="AF3" s="18"/>
+      <c r="AA3" s="19"/>
+      <c r="AB3" s="19"/>
+      <c r="AC3" s="19"/>
+      <c r="AD3" s="19"/>
+      <c r="AE3" s="19"/>
+      <c r="AF3" s="19"/>
     </row>
     <row r="4" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="J4" s="18" t="s">
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="J4" s="19" t="s">
         <v>3</v>
       </c>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
-      <c r="N4" s="18"/>
-      <c r="O4" s="18"/>
-      <c r="P4" s="18"/>
-      <c r="Q4" s="18"/>
-      <c r="R4" s="18"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
       <c r="Z4" s="3" t="s">
         <v>4</v>
       </c>
@@ -4341,36 +4408,36 @@
       </c>
     </row>
     <row r="11" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="19"/>
+      <c r="C11" s="18"/>
       <c r="D11" s="3" cm="1">
         <f t="array" aca="1" ref="D11" ca="1">INDIRECT("F" &amp; H11)</f>
         <v>0.3</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="19"/>
+      <c r="G11" s="18"/>
       <c r="H11" s="3">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="19"/>
+      <c r="C12" s="18"/>
       <c r="D12" s="5" cm="1">
         <f t="array" aca="1" ref="D12" ca="1">INDIRECT("E" &amp; H11)</f>
         <v>3.4375671399828902E-3</v>
       </c>
       <c r="E12" s="8"/>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="G12" s="19"/>
+      <c r="G12" s="18"/>
       <c r="H12" s="3" cm="1">
         <f t="array" aca="1" ref="H12" ca="1">IF(MAX(IF(C15:H15 &gt; D12, COLUMN(C15:H15)-COLUMN(C15)+1, 0))=0,3,MAX(IF(C15:H15 &gt; D12, COLUMN(C15:H15)-COLUMN(C15)+1, 0))+2)</f>
         <v>3</v>
@@ -4398,15 +4465,15 @@
       </c>
     </row>
     <row r="14" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
       <c r="K14" s="16" t="s">
         <v>27</v>
       </c>
@@ -4457,14 +4524,14 @@
       </c>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
+      <c r="G17" s="19"/>
       <c r="K17" s="16" t="s">
         <v>28</v>
       </c>
@@ -4476,10 +4543,10 @@
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B18" s="18" t="s">
+      <c r="B18" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="18"/>
+      <c r="C18" s="19"/>
       <c r="D18" s="9">
         <f ca="1">10^(_xlfn.FORECAST.LINEAR(D12,C6:D6,C15:D15))</f>
         <v>9.7292921327766527E-2</v>
@@ -4516,15 +4583,15 @@
       </c>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="17"/>
-      <c r="E21" s="17" t="s">
+      <c r="C21" s="20"/>
+      <c r="E21" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B22" s="3" t="s">
@@ -4753,12 +4820,12 @@
     <mergeCell ref="J4:R4"/>
   </mergeCells>
   <conditionalFormatting sqref="C15:H15">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
       <formula>$D$12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E23:E37">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>$D$12</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4780,17 +4847,17 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:15" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="G2" s="21" t="s">
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="G2" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="21"/>
-      <c r="I2" s="21"/>
-      <c r="J2" s="21"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
     </row>
     <row r="3" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B3" s="11" t="s">
@@ -4956,11 +5023,11 @@
       </c>
     </row>
     <row r="13" spans="2:15" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B13" s="20" t="s">
+      <c r="B13" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="21"/>
       <c r="M13" s="13">
         <v>40</v>
       </c>
@@ -5124,11 +5191,11 @@
       <c r="D23" s="12"/>
     </row>
     <row r="24" spans="2:14" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B24" s="20" t="s">
+      <c r="B24" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B25" s="11" t="s">

</xml_diff>

<commit_message>
Final codes to review process of filtering and extending simulation
</commit_message>
<xml_diff>
--- a/SSW_CurvaCalibracion.xlsx
+++ b/SSW_CurvaCalibracion.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pablo\Desktop\InvestigacionUSFQ\SSWCompleteAnalysis\SingleSolitaryWaveAnalysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{183DB95F-24AD-4F91-B687-735AA29AEF55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94A045B9-40BC-479E-814F-5446D060914D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{2BD432D8-4488-4A89-A586-01F393994D8E}"/>
   </bookViews>
   <sheets>
-    <sheet name="SSW_CalibrationCurve (2)" sheetId="4" r:id="rId1"/>
-    <sheet name="SSW_CalibrationCurve" sheetId="2" r:id="rId2"/>
-    <sheet name="K_values" sheetId="3" r:id="rId3"/>
+    <sheet name="SSW_Curve_Final" sheetId="5" r:id="rId1"/>
+    <sheet name="SSW_CalibrationCurve (2)" sheetId="4" r:id="rId2"/>
+    <sheet name="SSW_CalibrationCurve" sheetId="2" r:id="rId3"/>
+    <sheet name="K_values" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -60,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="37">
   <si>
     <t>Archivo: SSW_GroupSimulationModel.m</t>
   </si>
@@ -192,17 +193,24 @@
   <si>
     <t>0p40</t>
   </si>
+  <si>
+    <t>0.3 10 Mpa Sin K</t>
+  </si>
+  <si>
+    <t>0.5 10 Mpa Sin K</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.000000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.00000"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -252,6 +260,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -322,7 +336,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
@@ -349,10 +363,21 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="7" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -364,14 +389,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{A0AC99EA-4BF8-4951-9183-DBD917378CE6}"/>
     <cellStyle name="Normal 2 2" xfId="1" xr:uid="{C90D40CB-6B8A-4A17-91CD-8EF2FD126B89}"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -412,6 +436,16 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -439,45 +473,36 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="9.1803149606299206E-2"/>
+          <c:y val="5.0925925925925923E-2"/>
+          <c:w val="0.7620995188101487"/>
+          <c:h val="0.89814814814814814"/>
+        </c:manualLayout>
+      </c:layout>
       <c:scatterChart>
         <c:scatterStyle val="smoothMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>SSW_Curve_Final!$B$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0.5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="19050" cap="rnd">
               <a:solidFill>
@@ -504,54 +529,54 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'SSW_CalibrationCurve (2)'!$C$8:$H$8</c:f>
+              <c:f>SSW_Curve_Final!$C$5:$H$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>3.6903573000000001E-3</c:v>
+                  <c:v>3.6714E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.5245798642394099E-3</c:v>
+                  <c:v>3.4153E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.2349915672320801E-3</c:v>
+                  <c:v>3.2349000000000002E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.1210804794715E-3</c:v>
+                  <c:v>2.7461999999999999E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.0543159670394599E-3</c:v>
-                </c:pt>
-                <c:pt idx="5" formatCode="0.000000">
-                  <c:v>9.8983598711006393E-4</c:v>
+                  <c:v>2.5167000000000002E-3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.14970508462505E-3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SSW_CalibrationCurve (2)'!$C$5:$H$5</c:f>
+              <c:f>SSW_Curve_Final!$C$2:$H$2</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
                   <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>100</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>300</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>500</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>700</c:v>
-                </c:pt>
-                <c:pt idx="5" formatCode="General">
-                  <c:v>1000</c:v>
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="0.00">
+                  <c:v>10</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -559,13 +584,24 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-1EAD-4AA4-8D47-80FD66777F4A}"/>
+              <c16:uniqueId val="{00000000-BAD5-4BF1-B6BC-AA0BD3FFFA91}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>SSW_Curve_Final!$N$11</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0p30</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="19050" cap="rnd">
               <a:solidFill>
@@ -592,7 +628,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'SSW_CalibrationCurve (2)'!$E$23</c:f>
+              <c:f>SSW_Curve_Final!$O$11</c:f>
               <c:numCache>
                 <c:formatCode>0.00000</c:formatCode>
                 <c:ptCount val="1"/>
@@ -604,12 +640,12 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SSW_CalibrationCurve (2)'!$G$23</c:f>
+              <c:f>SSW_Curve_Final!$R$11</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
+                <c:formatCode>0.000</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>3.467614180219901</c:v>
+                  <c:v>7.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -617,13 +653,24 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-1FB9-4DFA-B9B0-A29027BAC4F9}"/>
+              <c16:uniqueId val="{00000001-BAD5-4BF1-B6BC-AA0BD3FFFA91}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="2"/>
           <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>SSW_Curve_Final!$N$12</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0p35</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
           <c:spPr>
             <a:ln w="19050" cap="rnd">
               <a:solidFill>
@@ -650,54 +697,24 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'SSW_CalibrationCurve (2)'!$C$9:$H$9</c:f>
+              <c:f>SSW_Curve_Final!$O$12</c:f>
               <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>3.6403573E-3</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1.4839440203368701E-3</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>1.19766476738336E-3</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.0891446262729801E-3</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.02655644409088E-3</c:v>
-                </c:pt>
-                <c:pt idx="5" formatCode="0.000000">
-                  <c:v>9.6648717426287402E-4</c:v>
+                  <c:v>3.3203773511161199E-3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'SSW_CalibrationCurve (2)'!$C$5:$H$5</c:f>
+              <c:f>SSW_Curve_Final!$Q$12</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0.1</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>300</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>500</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>700</c:v>
-                </c:pt>
-                <c:pt idx="5" formatCode="General">
-                  <c:v>1000</c:v>
+                  <c:v>5.56</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -705,7 +722,76 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-1FB9-4DFA-B9B0-A29027BAC4F9}"/>
+              <c16:uniqueId val="{00000002-BAD5-4BF1-B6BC-AA0BD3FFFA91}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>SSW_Curve_Final!$N$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0p40</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent4"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>SSW_Curve_Final!$O$13</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>3.4961620344202199E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>SSW_Curve_Final!$Q$13</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0.18</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-851C-43B2-AD2B-7E0699A08257}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -717,13 +803,14 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="1420178976"/>
-        <c:axId val="1420179936"/>
+        <c:axId val="317552319"/>
+        <c:axId val="317559519"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="1420178976"/>
+        <c:axId val="317552319"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:min val="2.0000000000000005E-3"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -778,14 +865,13 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1420179936"/>
+        <c:crossAx val="317559519"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1420179936"/>
+        <c:axId val="317559519"/>
         <c:scaling>
-          <c:logBase val="10"/>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -804,6 +890,575 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="317552319"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="103"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="3"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="8.8149736002717166E-2"/>
+          <c:y val="3.6436257545135187E-2"/>
+          <c:w val="0.87612213270007666"/>
+          <c:h val="0.88698709186240399"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Pois 0.30</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:shade val="53000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'SSW_CalibrationCurve (2)'!$C$8:$H$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>3.6903573000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.5245798642394099E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.2349915672320801E-3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.1210804794715E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.0543159670394599E-3</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="0.000000">
+                  <c:v>9.8983598711006393E-4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'SSW_CalibrationCurve (2)'!$C$5:$H$5</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="General">
+                  <c:v>1000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-1EAD-4AA4-8D47-80FD66777F4A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Pois 0.50</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'SSW_CalibrationCurve (2)'!$C$9:$H$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>3.6403573E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.4839440203368701E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.19766476738336E-3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.0891446262729801E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.02655644409088E-3</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="0.000000">
+                  <c:v>9.6648717426287402E-4</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'SSW_CalibrationCurve (2)'!$C$5:$H$5</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>700</c:v>
+                </c:pt>
+                <c:pt idx="5" formatCode="General">
+                  <c:v>1000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-1FB9-4DFA-B9B0-A29027BAC4F9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>0p30</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:shade val="76000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="diamond"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'SSW_CalibrationCurve (2)'!$E$23</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>2.5586437235105598E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'SSW_CalibrationCurve (2)'!$G$23</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>8.11</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-1FB9-4DFA-B9B0-A29027BAC4F9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:v>0p35</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="x"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="C00000"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'SSW_CalibrationCurve (2)'!$E$24</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>3.3203773511161199E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'SSW_CalibrationCurve (2)'!$G$24</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>5.56</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-6FED-469B-BC34-2B69605138F4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>0p40</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:tint val="54000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="0070C0"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="0070C0"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'SSW_CalibrationCurve (2)'!$E$25</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>3.4961620344202199E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'SSW_CalibrationCurve (2)'!$G$25</c:f>
+              <c:numCache>
+                <c:formatCode>0.000</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>0.18</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-6FED-469B-BC34-2B69605138F4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1420178976"/>
+        <c:axId val="1420179936"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1420178976"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="1.0000000000000002E-3"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="low"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1420179936"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1420179936"/>
+        <c:scaling>
+          <c:logBase val="10"/>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
         <c:numFmt formatCode="0.00" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -853,6 +1508,47 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.84601702345051888"/>
+          <c:y val="3.2331244964584845E-2"/>
+          <c:w val="0.12411298183738563"/>
+          <c:h val="0.28056094909545626"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
@@ -897,7 +1593,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -1428,6 +2124,12 @@
 </file>
 
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinear" id="14">
+  <a:schemeClr val="accent1"/>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -2499,20 +3201,577 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>249330</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>82364</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>349247</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>82097</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>386602</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>151280</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>380998</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>103868</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4B8706A8-66E3-3EA5-F1B8-67D33ADE36C8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>469597</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>70459</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>606869</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>139374</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2540,7 +3799,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
@@ -3274,6 +4533,288 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E91E2221-804C-494B-B283-F4CA5455FFE0}">
+  <dimension ref="B2:S13"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="16384" width="9.06640625" style="10"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:19" x14ac:dyDescent="0.45">
+      <c r="B2" s="21" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="E2" s="3">
+        <v>1</v>
+      </c>
+      <c r="F2" s="3">
+        <v>4</v>
+      </c>
+      <c r="G2" s="3">
+        <v>7</v>
+      </c>
+      <c r="H2" s="4">
+        <v>10</v>
+      </c>
+      <c r="I2" s="4">
+        <v>100</v>
+      </c>
+      <c r="J2" s="4">
+        <v>300</v>
+      </c>
+      <c r="K2" s="4">
+        <v>500</v>
+      </c>
+      <c r="L2" s="4">
+        <v>700</v>
+      </c>
+      <c r="M2" s="3">
+        <v>1000</v>
+      </c>
+      <c r="P2" s="10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="2:19" x14ac:dyDescent="0.45">
+      <c r="B3" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3">
+        <v>2.1252823576404498E-3</v>
+      </c>
+      <c r="I3" s="3">
+        <v>1.5349548257569E-3</v>
+      </c>
+      <c r="J3" s="3">
+        <v>1.2459906107288501E-3</v>
+      </c>
+      <c r="K3" s="3">
+        <v>1.13030798522664E-3</v>
+      </c>
+      <c r="L3" s="3">
+        <v>1.06244287429404E-3</v>
+      </c>
+      <c r="M3" s="5">
+        <v>9.978169398421491E-4</v>
+      </c>
+      <c r="P3" s="10">
+        <v>2.4484369999999999E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="2:19" x14ac:dyDescent="0.45">
+      <c r="B4" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="C4" s="3">
+        <v>3.6903573000000001E-3</v>
+      </c>
+      <c r="D4" s="3">
+        <v>3.4573999999999998E-3</v>
+      </c>
+      <c r="E4" s="3">
+        <v>3.2899280000000001E-3</v>
+      </c>
+      <c r="F4" s="3">
+        <v>2.8225659999999999E-3</v>
+      </c>
+      <c r="G4" s="3">
+        <v>2.597088E-3</v>
+      </c>
+      <c r="H4" s="3">
+        <v>2.15971893357225E-3</v>
+      </c>
+      <c r="I4" s="3">
+        <v>1.5245798642394099E-3</v>
+      </c>
+      <c r="J4" s="3">
+        <v>1.2349915672320801E-3</v>
+      </c>
+      <c r="K4" s="3">
+        <v>1.1210804794715E-3</v>
+      </c>
+      <c r="L4" s="3">
+        <v>1.0543159670394599E-3</v>
+      </c>
+      <c r="M4" s="5">
+        <v>9.8983598711006393E-4</v>
+      </c>
+      <c r="P4" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="2:19" x14ac:dyDescent="0.45">
+      <c r="B5" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="C5" s="3">
+        <v>3.6714E-3</v>
+      </c>
+      <c r="D5" s="3">
+        <v>3.4153E-3</v>
+      </c>
+      <c r="E5" s="3">
+        <v>3.2349000000000002E-3</v>
+      </c>
+      <c r="F5" s="3">
+        <v>2.7461999999999999E-3</v>
+      </c>
+      <c r="G5" s="3">
+        <v>2.5167000000000002E-3</v>
+      </c>
+      <c r="H5" s="3">
+        <v>2.14970508462505E-3</v>
+      </c>
+      <c r="I5" s="3">
+        <v>1.4839440203368701E-3</v>
+      </c>
+      <c r="J5" s="3">
+        <v>1.19766476738336E-3</v>
+      </c>
+      <c r="K5" s="3">
+        <v>1.0891446262729801E-3</v>
+      </c>
+      <c r="L5" s="3">
+        <v>1.02655644409088E-3</v>
+      </c>
+      <c r="M5" s="5">
+        <v>9.6648717426287402E-4</v>
+      </c>
+      <c r="P5" s="10">
+        <v>2.3674E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="2:19" x14ac:dyDescent="0.45">
+      <c r="B6" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="22">
+        <f>LOG(C2)</f>
+        <v>-1</v>
+      </c>
+      <c r="D6" s="22">
+        <f t="shared" ref="D6:M6" si="0">LOG(D2)</f>
+        <v>-0.3010299956639812</v>
+      </c>
+      <c r="E6" s="22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F6" s="22">
+        <f t="shared" si="0"/>
+        <v>0.6020599913279624</v>
+      </c>
+      <c r="G6" s="22">
+        <f t="shared" si="0"/>
+        <v>0.84509804001425681</v>
+      </c>
+      <c r="H6" s="22">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="I6" s="22">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="J6" s="22">
+        <f t="shared" si="0"/>
+        <v>2.4771212547196626</v>
+      </c>
+      <c r="K6" s="22">
+        <f t="shared" si="0"/>
+        <v>2.6989700043360187</v>
+      </c>
+      <c r="L6" s="22">
+        <f t="shared" si="0"/>
+        <v>2.8450980400142569</v>
+      </c>
+      <c r="M6" s="22">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="2:19" x14ac:dyDescent="0.45">
+      <c r="N11" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="O11" s="18">
+        <v>2.5586437235105598E-3</v>
+      </c>
+      <c r="P11" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="Q11" s="19">
+        <v>8.11</v>
+      </c>
+      <c r="R11" s="19">
+        <v>7.25</v>
+      </c>
+      <c r="S11" s="1">
+        <v>3.467614180219901</v>
+      </c>
+    </row>
+    <row r="12" spans="2:19" x14ac:dyDescent="0.45">
+      <c r="N12" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="O12" s="18">
+        <v>3.3203773511161199E-3</v>
+      </c>
+      <c r="P12" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="Q12" s="19">
+        <v>5.56</v>
+      </c>
+      <c r="R12" s="19">
+        <v>5.56</v>
+      </c>
+      <c r="S12" s="1">
+        <v>0.29870404899774289</v>
+      </c>
+    </row>
+    <row r="13" spans="2:19" x14ac:dyDescent="0.45">
+      <c r="N13" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="O13" s="18">
+        <v>3.4961620344202199E-3</v>
+      </c>
+      <c r="P13" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="Q13" s="19">
+        <v>0.18</v>
+      </c>
+      <c r="R13" s="19">
+        <v>0.18</v>
+      </c>
+      <c r="S13" s="1">
+        <v>0.16963693563959908</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="O11:O13">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+      <formula>$D$12</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{556E6EB9-EF01-4C35-8A8F-2C6A845001C7}">
   <dimension ref="B2:AF37"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -3297,37 +4838,37 @@
       </c>
     </row>
     <row r="3" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="Z3" s="19" t="s">
+      <c r="Z3" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="AA3" s="19"/>
-      <c r="AB3" s="19"/>
-      <c r="AC3" s="19"/>
-      <c r="AD3" s="19"/>
-      <c r="AE3" s="19"/>
-      <c r="AF3" s="19"/>
+      <c r="AA3" s="23"/>
+      <c r="AB3" s="23"/>
+      <c r="AC3" s="23"/>
+      <c r="AD3" s="23"/>
+      <c r="AE3" s="23"/>
+      <c r="AF3" s="23"/>
     </row>
     <row r="4" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="J4" s="19" t="s">
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="J4" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="23"/>
+      <c r="R4" s="23"/>
       <c r="Z4" s="3" t="s">
         <v>4</v>
       </c>
@@ -3379,7 +4920,7 @@
         <v>1</v>
       </c>
       <c r="L5" s="3">
-        <v>5</v>
+        <v>0.1</v>
       </c>
       <c r="M5" s="4">
         <v>10</v>
@@ -3458,7 +4999,7 @@
       </c>
       <c r="L6" s="4">
         <f>LOG10(L5)</f>
-        <v>0.69897000433601886</v>
+        <v>-1</v>
       </c>
       <c r="M6" s="4">
         <f>LOG10(M5)</f>
@@ -3518,7 +5059,9 @@
         <v>0.1</v>
       </c>
       <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
+      <c r="L7" s="3">
+        <v>3.7203573000000002E-3</v>
+      </c>
       <c r="M7" s="1">
         <v>2.1867939205959799E-3</v>
       </c>
@@ -3585,7 +5128,9 @@
         <v>0.3</v>
       </c>
       <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
+      <c r="L8" s="3">
+        <v>3.6903573000000001E-3</v>
+      </c>
       <c r="M8" s="3">
         <v>2.15971893357225E-3</v>
       </c>
@@ -3652,7 +5197,9 @@
         <v>0.5</v>
       </c>
       <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
+      <c r="L9" s="3">
+        <v>3.6403573E-3</v>
+      </c>
       <c r="M9" s="3">
         <v>2.14970508462505E-3</v>
       </c>
@@ -3673,36 +5220,36 @@
       </c>
     </row>
     <row r="11" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="18"/>
+      <c r="C11" s="24"/>
       <c r="D11" s="3" cm="1">
         <f t="array" aca="1" ref="D11" ca="1">INDIRECT("F" &amp; H11)</f>
         <v>0.5</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="18"/>
+      <c r="G11" s="24"/>
       <c r="H11" s="3">
         <v>25</v>
       </c>
     </row>
     <row r="12" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="18"/>
+      <c r="C12" s="24"/>
       <c r="D12" s="5" cm="1">
         <f t="array" aca="1" ref="D12" ca="1">INDIRECT("E" &amp; H11)</f>
         <v>3.4961620344202199E-3</v>
       </c>
       <c r="E12" s="8"/>
-      <c r="F12" s="18" t="s">
+      <c r="F12" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="G12" s="18"/>
+      <c r="G12" s="24"/>
       <c r="H12" s="3" cm="1">
         <f t="array" aca="1" ref="H12" ca="1">IF(MAX(IF(C15:H15 &gt; D12, COLUMN(C15:H15)-COLUMN(C15)+1, 0))=0,3,MAX(IF(C15:H15 &gt; D12, COLUMN(C15:H15)-COLUMN(C15)+1, 0))+2)</f>
         <v>3</v>
@@ -3733,15 +5280,15 @@
       </c>
     </row>
     <row r="14" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="19"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
       <c r="K14" s="16" t="s">
         <v>27</v>
       </c>
@@ -3792,14 +5339,14 @@
       </c>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
       <c r="K17" s="16" t="s">
         <v>28</v>
       </c>
@@ -3811,10 +5358,10 @@
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="19"/>
+      <c r="C18" s="23"/>
       <c r="D18" s="9">
         <f ca="1">10^(_xlfn.FORECAST.LINEAR(D12,C6:D6,C15:D15))</f>
         <v>0.16963693563959908</v>
@@ -3851,11 +5398,11 @@
       </c>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="E21" s="20" t="s">
+      <c r="E21" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="25"/>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.45">
       <c r="E22" s="3" t="s">
@@ -3878,44 +5425,62 @@
       </c>
     </row>
     <row r="23" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="E23" s="23">
+      <c r="E23" s="18">
         <v>2.5586437235105598E-3</v>
       </c>
       <c r="F23" s="3">
         <v>0.5</v>
       </c>
-      <c r="G23" s="3">
+      <c r="G23" s="19">
+        <v>8.11</v>
+      </c>
+      <c r="H23" s="19">
+        <v>7.25</v>
+      </c>
+      <c r="I23" s="1">
         <v>3.467614180219901</v>
       </c>
     </row>
     <row r="24" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="D24" s="1" t="s">
+      <c r="D24" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E24" s="23">
+      <c r="E24" s="18">
         <v>3.3203773511161199E-3</v>
       </c>
       <c r="F24" s="3">
         <v>0.5</v>
       </c>
-      <c r="G24" s="3">
+      <c r="G24" s="19">
+        <v>5.56</v>
+      </c>
+      <c r="H24" s="19">
+        <v>5.56</v>
+      </c>
+      <c r="I24" s="1">
         <v>0.29870404899774289</v>
       </c>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="D25" s="1" t="s">
+      <c r="D25" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="E25" s="23">
+      <c r="E25" s="18">
         <v>3.4961620344202199E-3</v>
       </c>
       <c r="F25" s="3">
         <v>0.5</v>
       </c>
-      <c r="G25" s="3">
+      <c r="G25" s="19">
+        <v>0.18</v>
+      </c>
+      <c r="H25" s="19">
+        <v>0.18</v>
+      </c>
+      <c r="I25" s="1">
         <v>0.16963693563959908</v>
       </c>
     </row>
@@ -4008,7 +5573,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80A9438D-FD9D-44C5-9D03-77FA3395C423}">
   <dimension ref="B2:AF37"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -4032,37 +5597,37 @@
       </c>
     </row>
     <row r="3" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="Z3" s="19" t="s">
+      <c r="Z3" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="AA3" s="19"/>
-      <c r="AB3" s="19"/>
-      <c r="AC3" s="19"/>
-      <c r="AD3" s="19"/>
-      <c r="AE3" s="19"/>
-      <c r="AF3" s="19"/>
+      <c r="AA3" s="23"/>
+      <c r="AB3" s="23"/>
+      <c r="AC3" s="23"/>
+      <c r="AD3" s="23"/>
+      <c r="AE3" s="23"/>
+      <c r="AF3" s="23"/>
     </row>
     <row r="4" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="J4" s="19" t="s">
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="J4" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
+      <c r="O4" s="23"/>
+      <c r="P4" s="23"/>
+      <c r="Q4" s="23"/>
+      <c r="R4" s="23"/>
       <c r="Z4" s="3" t="s">
         <v>4</v>
       </c>
@@ -4408,36 +5973,36 @@
       </c>
     </row>
     <row r="11" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="18"/>
+      <c r="C11" s="24"/>
       <c r="D11" s="3" cm="1">
         <f t="array" aca="1" ref="D11" ca="1">INDIRECT("F" &amp; H11)</f>
         <v>0.3</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="G11" s="18"/>
+      <c r="G11" s="24"/>
       <c r="H11" s="3">
         <v>23</v>
       </c>
     </row>
     <row r="12" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="C12" s="18"/>
+      <c r="C12" s="24"/>
       <c r="D12" s="5" cm="1">
         <f t="array" aca="1" ref="D12" ca="1">INDIRECT("E" &amp; H11)</f>
         <v>3.4375671399828902E-3</v>
       </c>
       <c r="E12" s="8"/>
-      <c r="F12" s="18" t="s">
+      <c r="F12" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="G12" s="18"/>
+      <c r="G12" s="24"/>
       <c r="H12" s="3" cm="1">
         <f t="array" aca="1" ref="H12" ca="1">IF(MAX(IF(C15:H15 &gt; D12, COLUMN(C15:H15)-COLUMN(C15)+1, 0))=0,3,MAX(IF(C15:H15 &gt; D12, COLUMN(C15:H15)-COLUMN(C15)+1, 0))+2)</f>
         <v>3</v>
@@ -4465,15 +6030,15 @@
       </c>
     </row>
     <row r="14" spans="2:32" x14ac:dyDescent="0.45">
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="19"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="23"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
       <c r="K14" s="16" t="s">
         <v>27</v>
       </c>
@@ -4524,14 +6089,14 @@
       </c>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="23"/>
       <c r="K17" s="16" t="s">
         <v>28</v>
       </c>
@@ -4543,10 +6108,10 @@
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C18" s="19"/>
+      <c r="C18" s="23"/>
       <c r="D18" s="9">
         <f ca="1">10^(_xlfn.FORECAST.LINEAR(D12,C6:D6,C15:D15))</f>
         <v>9.7292921327766527E-2</v>
@@ -4583,15 +6148,15 @@
       </c>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B21" s="20" t="s">
+      <c r="B21" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="20"/>
-      <c r="E21" s="20" t="s">
+      <c r="C21" s="25"/>
+      <c r="E21" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="25"/>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B22" s="3" t="s">
@@ -4833,7 +6398,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D0AE93B-6E63-4919-B10E-28F208192998}">
   <dimension ref="B2:O33"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -4847,17 +6412,17 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:15" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="G2" s="22" t="s">
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="G2" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
     </row>
     <row r="3" spans="2:15" x14ac:dyDescent="0.45">
       <c r="B3" s="11" t="s">
@@ -5023,11 +6588,11 @@
       </c>
     </row>
     <row r="13" spans="2:15" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
       <c r="M13" s="13">
         <v>40</v>
       </c>
@@ -5191,11 +6756,11 @@
       <c r="D23" s="12"/>
     </row>
     <row r="24" spans="2:14" ht="15.75" x14ac:dyDescent="0.5">
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="26"/>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B25" s="11" t="s">

</xml_diff>